<commit_message>
docs: new scope of project
</commit_message>
<xml_diff>
--- a/data_samples/Datos_Entrada.xlsx
+++ b/data_samples/Datos_Entrada.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24729"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyecto PSO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\optimizacion-embalses\data_samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4DC011-DE4F-4077-8FF3-0FB8662C6B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92CFC1D9-3562-4811-833E-727F9705639C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -677,7 +677,7 @@
         <v>100</v>
       </c>
       <c r="C2">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F2" s="5">
         <v>2.0833333333333332E-2</v>
@@ -730,7 +730,7 @@
         <v>100</v>
       </c>
       <c r="C3">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F3" s="5">
         <v>4.1666666666666664E-2</v>
@@ -783,7 +783,7 @@
         <v>100</v>
       </c>
       <c r="C4">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F4" s="5">
         <v>6.25E-2</v>
@@ -833,10 +833,10 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="C5">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F5" s="5">
         <v>8.3333333333333329E-2</v>
@@ -886,10 +886,10 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="C6">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F6" s="5">
         <v>0.104166666666667</v>
@@ -939,10 +939,10 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="C7">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F7" s="5">
         <v>0.125</v>
@@ -992,10 +992,10 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="C8">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F8" s="5">
         <v>0.14583333333333301</v>
@@ -1045,10 +1045,10 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="C9">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F9" s="5">
         <v>0.16666666666666599</v>
@@ -1098,10 +1098,10 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="C10">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F10" s="5">
         <v>0.1875</v>
@@ -1151,10 +1151,10 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="C11">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="F11" s="5">
         <v>0.20833333333333301</v>
@@ -1204,10 +1204,10 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="C12">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F12" s="5">
         <v>0.22916666666666599</v>
@@ -1257,10 +1257,10 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="C13">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F13" s="5">
         <v>0.25</v>
@@ -1310,10 +1310,10 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="C14">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="F14" s="5">
         <v>0.27083333333333298</v>
@@ -1363,10 +1363,10 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="C15">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="F15" s="5">
         <v>0.29166666666666602</v>
@@ -1419,7 +1419,7 @@
         <v>200</v>
       </c>
       <c r="C16">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="F16" s="5">
         <v>0.3125</v>
@@ -1472,7 +1472,7 @@
         <v>200</v>
       </c>
       <c r="C17">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="F17" s="5">
         <v>0.33333333333333298</v>
@@ -1525,7 +1525,7 @@
         <v>200</v>
       </c>
       <c r="C18">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="F18" s="5">
         <v>0.35416666666666602</v>
@@ -1578,7 +1578,7 @@
         <v>200</v>
       </c>
       <c r="C19">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="F19" s="5">
         <v>0.375</v>
@@ -1631,7 +1631,7 @@
         <v>200</v>
       </c>
       <c r="C20">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="F20" s="5">
         <v>0.39583333333333298</v>
@@ -1681,10 +1681,10 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="C21">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="F21" s="5">
         <v>0.41666666666666602</v>
@@ -1734,10 +1734,10 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="C22">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="F22" s="5">
         <v>0.4375</v>
@@ -1787,10 +1787,10 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="C23">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="F23" s="5">
         <v>0.45833333333333298</v>
@@ -1840,10 +1840,10 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="C24">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="F24" s="5">
         <v>0.47916666666666602</v>
@@ -1893,10 +1893,10 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="C25">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="F25" s="5">
         <v>0.5</v>
@@ -1946,10 +1946,10 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="C26">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="F26" s="5">
         <v>0.52083333333333304</v>
@@ -1999,10 +1999,10 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="C27">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F27" s="5">
         <v>0.54166666666666596</v>
@@ -2055,7 +2055,7 @@
         <v>200</v>
       </c>
       <c r="C28">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F28" s="5">
         <v>0.5625</v>
@@ -2108,7 +2108,7 @@
         <v>200</v>
       </c>
       <c r="C29">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F29" s="5">
         <v>0.58333333333333304</v>
@@ -2161,7 +2161,7 @@
         <v>200</v>
       </c>
       <c r="C30">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F30" s="5">
         <v>0.60416666666666596</v>
@@ -2214,7 +2214,7 @@
         <v>200</v>
       </c>
       <c r="C31">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F31" s="5">
         <v>0.625</v>
@@ -2320,7 +2320,7 @@
         <v>200</v>
       </c>
       <c r="C33">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F33" s="5">
         <v>0.66666666666666596</v>
@@ -2373,7 +2373,7 @@
         <v>200</v>
       </c>
       <c r="C34">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F34" s="5">
         <v>0.6875</v>
@@ -2426,7 +2426,7 @@
         <v>200</v>
       </c>
       <c r="C35">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F35" s="5">
         <v>0.70833333333333304</v>
@@ -2479,7 +2479,7 @@
         <v>200</v>
       </c>
       <c r="C36">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F36" s="5">
         <v>0.72916666666666596</v>
@@ -2529,10 +2529,10 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C37">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F37" s="5">
         <v>0.75</v>
@@ -2582,10 +2582,10 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C38">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="F38" s="5">
         <v>0.77083333333333304</v>
@@ -2635,10 +2635,10 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C39">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="F39" s="5">
         <v>0.79166666666666596</v>
@@ -2688,10 +2688,10 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C40">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="F40" s="5">
         <v>0.8125</v>
@@ -2741,10 +2741,10 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C41">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="F41" s="5">
         <v>0.83333333333333304</v>
@@ -2794,10 +2794,10 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C42">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="F42" s="5">
         <v>0.85416666666666596</v>
@@ -2847,7 +2847,7 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="C43">
         <v>100</v>
@@ -2900,10 +2900,10 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="C44">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F44" s="5">
         <v>0.89583333333333304</v>
@@ -2953,10 +2953,10 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="C45">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="F45" s="5">
         <v>0.91666666666666596</v>
@@ -3006,10 +3006,10 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="C46">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="F46" s="5">
         <v>0.9375</v>
@@ -3062,7 +3062,7 @@
         <v>100</v>
       </c>
       <c r="C47">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="F47" s="5">
         <v>0.95833333333333304</v>
@@ -3115,7 +3115,7 @@
         <v>100</v>
       </c>
       <c r="C48">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="F48" s="5">
         <v>0.97916666666666596</v>
@@ -3168,7 +3168,7 @@
         <v>100</v>
       </c>
       <c r="C49">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="F49" s="5">
         <v>1</v>
@@ -3216,7 +3216,7 @@
     <row r="50" spans="1:20">
       <c r="C50">
         <f>+SUM(C2:C49)/2</f>
-        <v>1867.5</v>
+        <v>1717.5</v>
       </c>
       <c r="G50">
         <f>+SUM(G2:G49)/2</f>
@@ -3254,7 +3254,7 @@
     <row r="51" spans="1:20">
       <c r="C51" s="3">
         <f>+C50/1.66189/24/3.6</f>
-        <v>13.006025268419288</v>
+        <v>11.961364604289226</v>
       </c>
       <c r="G51" s="6">
         <f>+G50/1.66189/24/3.6</f>
@@ -3293,7 +3293,7 @@
     <row r="52" spans="1:20">
       <c r="C52" s="4">
         <f>+ROUND(C51,1)</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G52">
         <f>+ROUND(G51,1)</f>

</xml_diff>